<commit_message>
benchmarks(joints): rj012, rj014 and rj019 declare the K0 their new tags name
A corpus file has to carry the K0 initial stress its test tag declares
(benchmarks/tag_k0.py, and run_tests.py's tag_k0 row). Problems 12, 14 and 19
carried no tag until this round, so their builders wrote no K0; now that the
three rows lock, the builder reads k0=1 off each tag and the files declare it.

The factor cannot move: the suite passes k0 to solve_ssrm as a keyword, so both
the old and the new file solve at K0 = 1. verify_rebuild.py --group joints is
back to 23/23 and the tag_k0 row passes.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj012.xlsx
+++ b/docs/verification/files/rocscience/joints/rj012.xlsx
@@ -3374,7 +3374,9 @@
       <c r="G16" t="s">
         <v>34</v>
       </c>
-      <c r="D16"/>
+      <c r="D16">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>

</xml_diff>